<commit_message>
docs: adopt the official Reading Taxonomy v1 workbook, drop the TR-01 override
The reissued workbook states its own status (Categories DECIDED, Skills
DECIDED v1) and carries the corrected rules directly: TR-01 now requires
exactly one Primary Skill, TR-02 states that a Secondary produces no
equal-weight mastery evidence, TR-10 makes the 50-100 question pilot optional
rather than a freeze gate, and a new TR-11 forbids parsing a skill code to
derive its Category.

That removes the temporary exception where this document overrode the workbook
on TR-01. Markdown and workbook now agree in full.

All 25 skill codes are unchanged between the two workbook revisions, which is
what the opaque-identifier rule requires once evidence can be attached.

CSV extracts regenerated and verified cell-by-cell against the workbook.

Document cleanup only: no table, no SQL, no migration, no seed, no frontend, no
Production change.
</commit_message>
<xml_diff>
--- a/docs/learn/reading-taxonomy/Reading_Taxonomy_v1.xlsx
+++ b/docs/learn/reading-taxonomy/Reading_Taxonomy_v1.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R9557c5d3b6e745e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category_Summary" sheetId="2" r:id="Rebc9fa74bb2d4208"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill_Taxonomy" sheetId="3" r:id="R51b233605e254069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tagging_Rules" sheetId="4" r:id="R0a2db4ee14f74101"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R74180b5354664556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category_Summary" sheetId="2" r:id="Refb992a7657c4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill_Taxonomy" sheetId="3" r:id="R22b5dfcc07404189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tagging_Rules" sheetId="4" r:id="R109e24ca839d4f1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +59,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -100,6 +100,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -308,7 +309,7 @@
   <x:sheetData>
     <x:row r="1" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>Reading Taxonomy v1 Candidate</x:v>
+        <x:v>Reading Taxonomy v1</x:v>
       </x:c>
       <x:c r="B1" s="14" t="str"/>
     </x:row>
@@ -325,7 +326,7 @@
         <x:v>層級</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>Domain → Category → Skill。Reading v1 暫時不建立 Micro-skill。</x:v>
+        <x:v>Domain → Category → Skill。Reading v1 不建立 Micro-skill。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -357,7 +358,7 @@
         <x:v>核心原則 1</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
-        <x:v>每一道可計分 Reading 題目至少標一個 Primary Skill。</x:v>
+        <x:v>每一道可計分 Reading assessable item 必須恰好標一個 Primary Skill。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -365,7 +366,7 @@
         <x:v>核心原則 2</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
-        <x:v>Secondary Skill 為 optional；只有題目真的同時測第二能力時才標，不因主題相關就固定雙標。</x:v>
+        <x:v>Secondary Skill 為 optional；預設不標。只有題目真的同時測第二能力時才標，且 v1 不自動產生與 Primary 等權的 mastery evidence。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -389,7 +390,7 @@
         <x:v>核心原則 5</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Skill code 是穩定識別碼；中文/英文顯示名稱未來可調整，但 code 一旦開始掛 evidence 不應輕易變更。</x:v>
+        <x:v>Skill code 是 stable opaque identifier；中文／英文顯示名稱未來可調整。任何程式不得 parse code 來推導 Category，Skill → Category 必須使用正式 taxonomy relationship。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -397,7 +398,7 @@
         <x:v>Validation</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
-        <x:v>正式 freeze 前，建議拿 50–100 題既有 Reading 題目做 AI-assisted pilot tagging，檢查是否能穩定落到單一 Primary Skill。</x:v>
+        <x:v>50–100 題既有 Reading 題目 pilot 可作為 OPTIONAL future validation；不是 v1 freeze gate 或 prerequisite。未來若需調整，以 v1.1 / v2 versioning 處理。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -405,7 +406,7 @@
         <x:v>狀態</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
-        <x:v>CANDIDATE；六大 Category 可視為 owner-approved 方向，25 個 Skill 尚待真題 pilot 驗證後 freeze。</x:v>
+        <x:v>DECIDED v1（2026-08-29）：6 Categories 與 25 Skills 已 freeze。Reading v1 不建立 Micro-skill。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -462,7 +463,7 @@
         <x:v>理解全文或段落的核心內容、摘要與主題訊息。</x:v>
       </x:c>
       <x:c r="F2" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -482,7 +483,7 @@
         <x:v>從文章中定位、配對與整合明示資訊與支持證據。</x:v>
       </x:c>
       <x:c r="F3" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -502,7 +503,7 @@
         <x:v>依上下文判斷字詞、表達、指涉與比喻／慣用意義。</x:v>
       </x:c>
       <x:c r="F4" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -522,7 +523,7 @@
         <x:v>根據文本證據推出未直接明說的資訊、原因、結論或意涵。</x:v>
       </x:c>
       <x:c r="F5" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -542,7 +543,7 @@
         <x:v>理解文章組織、句段功能、銜接關係與篇章排序。</x:v>
       </x:c>
       <x:c r="F6" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -562,7 +563,7 @@
         <x:v>判斷作者目的、態度、立場、修辭策略、文體與讀者。</x:v>
       </x:c>
       <x:c r="F7" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -640,7 +641,7 @@
         <x:v>不等同 Best Title 題型；若題目只是找某一段主旨，改標 Paragraph Main Idea</x:v>
       </x:c>
       <x:c r="I2" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -669,7 +670,7 @@
         <x:v>若問某段在全文中的功能，優先考慮 R5 Sentence &amp; Paragraph Function</x:v>
       </x:c>
       <x:c r="I3" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -698,7 +699,7 @@
         <x:v>若只是選出單一中心思想而非摘要多個重點，可標 Passage Central Idea</x:v>
       </x:c>
       <x:c r="I4" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -727,7 +728,7 @@
         <x:v>不要與作者寫作目的混同；Purpose 問的是作者為什麼寫</x:v>
       </x:c>
       <x:c r="I5" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -756,7 +757,7 @@
         <x:v>如果答案需要推出未明說的結論，改標 Inference</x:v>
       </x:c>
       <x:c r="I6" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -785,7 +786,7 @@
         <x:v>不只是答對內容，也要求定位支持依據</x:v>
       </x:c>
       <x:c r="I7" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -814,7 +815,7 @@
         <x:v>若需跨多處資訊再推出新結論，改標 Integration 或 Inference</x:v>
       </x:c>
       <x:c r="I8" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -843,7 +844,7 @@
         <x:v>A+B 仍只是文本已明說內容 → 本 Skill；A+B 推出未明說 C → Inference</x:v>
       </x:c>
       <x:c r="I9" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -872,7 +873,7 @@
         <x:v>不是單純脫離文本的字彙知識測驗</x:v>
       </x:c>
       <x:c r="I10" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -901,7 +902,7 @@
         <x:v>若主要考 figurative / idiomatic 特殊意義，可標 Figurative &amp; Idiomatic Meaning</x:v>
       </x:c>
       <x:c r="I11" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -930,7 +931,7 @@
         <x:v>重點是 antecedent/reference，不是一般 Grammar pronoun 題</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -959,7 +960,7 @@
         <x:v>若只是一般片語的語境字義，標 Phrase &amp; Expression Meaning</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -988,7 +989,7 @@
         <x:v>若需整合全文多段，標 Global Inference &amp; Conclusion</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1017,7 +1018,7 @@
         <x:v>若主要在判斷作者態度，優先標 R6 Tone &amp; Attitude</x:v>
       </x:c>
       <x:c r="I15" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -1046,7 +1047,7 @@
         <x:v>如果原因已直接寫出，標 Explicit Detail</x:v>
       </x:c>
       <x:c r="I16" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1075,7 +1076,7 @@
         <x:v>重點是文本沒有直接說出的 implication / prediction</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1104,7 +1105,7 @@
         <x:v>若題目問某一句/某一段在文中的作用，標 Function</x:v>
       </x:c>
       <x:c r="I18" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -1133,7 +1134,7 @@
         <x:v>不是作者整篇文章的目的；整篇 Purpose 歸 R6</x:v>
       </x:c>
       <x:c r="I19" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -1162,7 +1163,7 @@
         <x:v>若只是單純考某連接詞文法，可屬 Grammar，不是 Reading evidence</x:v>
       </x:c>
       <x:c r="I20" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -1191,7 +1192,7 @@
         <x:v>這不是單純 question type；真正能力是 discourse flow</x:v>
       </x:c>
       <x:c r="I21" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -1220,7 +1221,7 @@
         <x:v>不要與某句/某段的局部功能混同，後者通常是 R5 Function</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -1249,7 +1250,7 @@
         <x:v>雖常需推論，但 taxonomy 中 primary 固定歸 Purpose &amp; Style</x:v>
       </x:c>
       <x:c r="I23" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -1278,7 +1279,7 @@
         <x:v>若只是從全文推論一般結論、不涉及立場，標 Inference</x:v>
       </x:c>
       <x:c r="I24" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -1307,7 +1308,7 @@
         <x:v>若題目只問某段扮演什麼結構功能，可標 R5 Function</x:v>
       </x:c>
       <x:c r="I25" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -1336,7 +1337,7 @@
         <x:v>不等同 Tone；Tone 側重態度，Style/Register 側重表達方式與受眾</x:v>
       </x:c>
       <x:c r="I26" s="16" t="str">
-        <x:v>CANDIDATE</x:v>
+        <x:v>DECIDED v1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1369,21 +1370,21 @@
         <x:v>TR-01</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>每道可計分 Reading 題目至少一個 Primary Skill。</x:v>
+        <x:v>每一道可計分 Reading assessable item 必須恰好有一個 Primary Skill。</x:v>
       </x:c>
       <x:c r="C2" s="16" t="str">
-        <x:v>Q: What can be inferred...? → READ_INFER_*</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+        <x:v>Q: What can be inferred...? → 選一個最直接決定答對與否的 READ_INFER_* 作 Primary。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="16" t="str">
         <x:v>TR-02</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>Secondary Skill 是 optional，預設 null。只有題目真的同時測第二能力時才標。</x:v>
+        <x:v>Secondary Skill 是 optional，預設 null。只有題目真的同時測第二能力時才標；v1 不自動產生與 Primary Skill 等權的 mastery evidence。</x:v>
       </x:c>
       <x:c r="C3" s="16" t="str">
-        <x:v>不要因為 Context 題需要『推一下』就自動加 Inference secondary。</x:v>
+        <x:v>Secondary 先作 tagging / analysis metadata；不要因概念相關就固定雙標。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1446,10 +1447,10 @@
         <x:v>TR-08</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
-        <x:v>Reading v1 暫時不建立 Micro-skill。</x:v>
+        <x:v>Reading v1 不建立 Micro-skill。</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
-        <x:v>先驗證 25 Skills 是否足以穩定分類既有真題。</x:v>
+        <x:v>四層 taxonomy 是上限，不是配額；Reading v1 在 Skill 層結束是刻意設計。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1468,10 +1469,21 @@
         <x:v>TR-10</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>建議 pilot：先跑 50–100 題；若兩個 Skills 長期無法穩定區分，再合併或重命名。</x:v>
+        <x:v>50–100 題 pilot 是 OPTIONAL future validation，不是 freeze gate。</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
-        <x:v>taxonomy 用真題驗證，不先追求理論上的極細分類。</x:v>
+        <x:v>未來若實際使用後發現兩個 Skills 長期難以區分，可在 v1.1 / v2 合併、改名或調整。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="16" t="str">
+        <x:v>TR-11</x:v>
+      </x:c>
+      <x:c r="B12" s="16" t="str">
+        <x:v>Skill code 是 stable opaque identifier；禁止 parse code 字串來推導 Category。</x:v>
+      </x:c>
+      <x:c r="C12" s="16" t="str">
+        <x:v>READ_PURPOSE_TONE 屬 R6 必須由正式 taxonomy relationship 取得，不可從字串解析。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>